<commit_message>
Made the ALU and CU Testbenches
</commit_message>
<xml_diff>
--- a/Practical-3/MPI/compiled_benchmarks_mpi.xlsx
+++ b/Practical-3/MPI/compiled_benchmarks_mpi.xlsx
@@ -1,20 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29930"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uctcloud-my.sharepoint.com/personal/almmoh017_myuct_ac_za/Documents/Year 4/EEE4120F/EEE4120F_Practicals_Group10/Practical-3/MPI/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_BCD245B85A4E2E97D91C872A3AAE46FB91B9A647" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{346658B4-BF0E-4AF3-8ABB-96E509EF757A}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="22">
   <si>
     <t>Input</t>
   </si>
@@ -37,43 +59,46 @@
     <t>Best Path</t>
   </si>
   <si>
+    <t>Speedup</t>
+  </si>
+  <si>
     <t>energy4</t>
   </si>
   <si>
+    <t>1 4 2 3</t>
+  </si>
+  <si>
     <t>energy5</t>
   </si>
   <si>
+    <t>1 4 5 2 3</t>
+  </si>
+  <si>
     <t>energy6</t>
   </si>
   <si>
+    <t>1 4 6 5 2 3</t>
+  </si>
+  <si>
     <t>energy7</t>
   </si>
   <si>
+    <t>1 4 6 5 3 2 7</t>
+  </si>
+  <si>
     <t>energy8</t>
   </si>
   <si>
+    <t>1 4 6 5 8 3 2 7</t>
+  </si>
+  <si>
     <t>energy9</t>
   </si>
   <si>
+    <t>1 4 9 6 5 8 3 2 7</t>
+  </si>
+  <si>
     <t>energy10</t>
-  </si>
-  <si>
-    <t>1 4 2 3</t>
-  </si>
-  <si>
-    <t>1 4 5 2 3</t>
-  </si>
-  <si>
-    <t>1 4 6 5 2 3</t>
-  </si>
-  <si>
-    <t>1 4 6 5 3 2 7</t>
-  </si>
-  <si>
-    <t>1 4 6 5 8 3 2 7</t>
-  </si>
-  <si>
-    <t>1 4 9 6 5 8 3 2 7</t>
   </si>
   <si>
     <t>1 10 4 9 6 5 8 3 2 7</t>
@@ -82,7 +107,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -108,7 +133,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -131,13 +156,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -146,13 +185,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -190,7 +237,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -224,6 +271,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -258,9 +306,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -433,11 +482,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G50"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H50"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
+  <cols>
+    <col min="4" max="4" width="19.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -459,79 +512,82 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2">
-        <v>0.26413703</v>
+        <v>0.26413702999999999</v>
       </c>
       <c r="D2">
-        <v>9.799E-05</v>
+        <v>9.7990000000000002E-5</v>
       </c>
       <c r="E2">
-        <v>0.26423502</v>
+        <v>0.26423501999999999</v>
       </c>
       <c r="F2">
         <v>105</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3">
-        <v>0.23379493</v>
+        <v>0.23379493000000001</v>
       </c>
       <c r="D3">
-        <v>3.481E-05</v>
+        <v>3.481E-5</v>
       </c>
       <c r="E3">
-        <v>0.23382974</v>
+        <v>0.23382974000000001</v>
       </c>
       <c r="F3">
         <v>105</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B4">
         <v>4</v>
       </c>
       <c r="C4">
-        <v>0.25362396</v>
+        <v>0.25362395999999998</v>
       </c>
       <c r="D4">
-        <v>2.098E-05</v>
+        <v>2.0979999999999999E-5</v>
       </c>
       <c r="E4">
-        <v>0.25364494</v>
+        <v>0.25364493999999999</v>
       </c>
       <c r="F4">
         <v>105</v>
       </c>
       <c r="G4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5">
         <v>6</v>
@@ -540,136 +596,136 @@
         <v>0.2753911</v>
       </c>
       <c r="D5">
-        <v>0.00024891</v>
+        <v>2.4890999999999997E-4</v>
       </c>
       <c r="E5">
-        <v>0.27564001</v>
+        <v>0.27564000999999999</v>
       </c>
       <c r="F5">
         <v>105</v>
       </c>
       <c r="G5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>8</v>
       </c>
       <c r="C6">
-        <v>0.26377511</v>
+        <v>0.26377510999999998</v>
       </c>
       <c r="D6">
-        <v>4.101E-05</v>
+        <v>4.1010000000000002E-5</v>
       </c>
       <c r="E6">
-        <v>0.26381612</v>
+        <v>0.26381611999999999</v>
       </c>
       <c r="F6">
         <v>105</v>
       </c>
       <c r="G6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>10</v>
       </c>
       <c r="C7">
-        <v>0.27092981</v>
+        <v>0.27092980999999999</v>
       </c>
       <c r="D7">
-        <v>0.00023603</v>
+        <v>2.3603E-4</v>
       </c>
       <c r="E7">
-        <v>0.27116584</v>
+        <v>0.27116583999999999</v>
       </c>
       <c r="F7">
         <v>105</v>
       </c>
       <c r="G7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8">
         <v>12</v>
       </c>
       <c r="C8">
-        <v>0.29231882</v>
+        <v>0.29231881999999998</v>
       </c>
       <c r="D8">
-        <v>0.0001328</v>
+        <v>1.328E-4</v>
       </c>
       <c r="E8">
-        <v>0.29245162</v>
+        <v>0.29245162000000002</v>
       </c>
       <c r="F8">
         <v>105</v>
       </c>
       <c r="G8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9">
-        <v>0.22741795</v>
+        <v>0.22741795000000001</v>
       </c>
       <c r="D9">
-        <v>2.813E-05</v>
+        <v>2.813E-5</v>
       </c>
       <c r="E9">
-        <v>0.22744608</v>
+        <v>0.22744607999999999</v>
       </c>
       <c r="F9">
         <v>115</v>
       </c>
       <c r="G9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10">
-        <v>0.22981596</v>
+        <v>0.22981596000000001</v>
       </c>
       <c r="D10">
-        <v>1.502E-05</v>
+        <v>1.502E-5</v>
       </c>
       <c r="E10">
-        <v>0.22983098</v>
+        <v>0.22983097999999999</v>
       </c>
       <c r="F10">
         <v>115</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B11">
         <v>4</v>
@@ -678,90 +734,90 @@
         <v>0.24578595</v>
       </c>
       <c r="D11">
-        <v>2.408E-05</v>
+        <v>2.408E-5</v>
       </c>
       <c r="E11">
-        <v>0.24581003</v>
+        <v>0.24581003000000001</v>
       </c>
       <c r="F11">
         <v>115</v>
       </c>
       <c r="G11" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B12">
         <v>6</v>
       </c>
       <c r="C12">
-        <v>0.25613093</v>
+        <v>0.25613092999999998</v>
       </c>
       <c r="D12">
-        <v>4.196E-05</v>
+        <v>4.1959999999999998E-5</v>
       </c>
       <c r="E12">
-        <v>0.25617289</v>
+        <v>0.25617288999999999</v>
       </c>
       <c r="F12">
         <v>115</v>
       </c>
       <c r="G12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B13">
         <v>8</v>
       </c>
       <c r="C13">
-        <v>0.27558208</v>
+        <v>0.27558208000000001</v>
       </c>
       <c r="D13">
-        <v>3.314E-05</v>
+        <v>3.3139999999999998E-5</v>
       </c>
       <c r="E13">
-        <v>0.27561522</v>
+        <v>0.27561521999999999</v>
       </c>
       <c r="F13">
         <v>115</v>
       </c>
       <c r="G13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B14">
         <v>10</v>
       </c>
       <c r="C14">
-        <v>0.27110291</v>
+        <v>0.27110290999999997</v>
       </c>
       <c r="D14">
-        <v>8.297E-05</v>
+        <v>8.297E-5</v>
       </c>
       <c r="E14">
-        <v>0.27118588</v>
+        <v>0.27118587999999999</v>
       </c>
       <c r="F14">
         <v>115</v>
       </c>
       <c r="G14" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B15">
         <v>12</v>
@@ -770,44 +826,44 @@
         <v>0.28444099</v>
       </c>
       <c r="D15">
-        <v>6.509E-05</v>
+        <v>6.5090000000000002E-5</v>
       </c>
       <c r="E15">
-        <v>0.28450608</v>
+        <v>0.28450607999999999</v>
       </c>
       <c r="F15">
         <v>115</v>
       </c>
       <c r="G15" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16">
-        <v>0.22422004</v>
+        <v>0.22422004000000001</v>
       </c>
       <c r="D16">
-        <v>2.503E-05</v>
+        <v>2.5029999999999999E-5</v>
       </c>
       <c r="E16">
-        <v>0.22424507</v>
+        <v>0.22424506999999999</v>
       </c>
       <c r="F16">
         <v>124</v>
       </c>
       <c r="G16" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B17">
         <v>2</v>
@@ -816,7 +872,7 @@
         <v>0.22951794</v>
       </c>
       <c r="D17">
-        <v>1.979E-05</v>
+        <v>1.9789999999999999E-5</v>
       </c>
       <c r="E17">
         <v>0.22953773</v>
@@ -825,35 +881,35 @@
         <v>124</v>
       </c>
       <c r="G17" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B18">
         <v>4</v>
       </c>
       <c r="C18">
-        <v>0.244596</v>
+        <v>0.24459600000000001</v>
       </c>
       <c r="D18">
-        <v>2.789E-05</v>
+        <v>2.7889999999999999E-5</v>
       </c>
       <c r="E18">
-        <v>0.24462389</v>
+        <v>0.24462389000000001</v>
       </c>
       <c r="F18">
         <v>124</v>
       </c>
       <c r="G18" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B19">
         <v>6</v>
@@ -862,30 +918,30 @@
         <v>0.24932504</v>
       </c>
       <c r="D19">
-        <v>0.00022793</v>
+        <v>2.2792999999999999E-4</v>
       </c>
       <c r="E19">
-        <v>0.24955297</v>
+        <v>0.24955297000000001</v>
       </c>
       <c r="F19">
         <v>124</v>
       </c>
       <c r="G19" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B20">
         <v>8</v>
       </c>
       <c r="C20">
-        <v>0.2681489</v>
+        <v>0.26814890000000002</v>
       </c>
       <c r="D20">
-        <v>3.886E-05</v>
+        <v>3.8859999999999997E-5</v>
       </c>
       <c r="E20">
         <v>0.26818776</v>
@@ -894,58 +950,58 @@
         <v>124</v>
       </c>
       <c r="G20" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B21">
         <v>10</v>
       </c>
       <c r="C21">
-        <v>0.26756811</v>
+        <v>0.26756811000000003</v>
       </c>
       <c r="D21">
-        <v>0.00031304</v>
+        <v>3.1304E-4</v>
       </c>
       <c r="E21">
-        <v>0.26788115</v>
+        <v>0.26788115000000001</v>
       </c>
       <c r="F21">
         <v>124</v>
       </c>
       <c r="G21" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B22">
         <v>12</v>
       </c>
       <c r="C22">
-        <v>0.28244615</v>
+        <v>0.28244615000000001</v>
       </c>
       <c r="D22">
-        <v>5.007E-05</v>
+        <v>5.007E-5</v>
       </c>
       <c r="E22">
-        <v>0.28249622</v>
+        <v>0.28249622000000002</v>
       </c>
       <c r="F22">
         <v>124</v>
       </c>
       <c r="G22" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B23">
         <v>1</v>
@@ -954,7 +1010,7 @@
         <v>0.22375202</v>
       </c>
       <c r="D23">
-        <v>2.789E-05</v>
+        <v>2.7889999999999999E-5</v>
       </c>
       <c r="E23">
         <v>0.22377991</v>
@@ -963,12 +1019,12 @@
         <v>145</v>
       </c>
       <c r="G23" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B24">
         <v>2</v>
@@ -977,44 +1033,44 @@
         <v>0.23192883</v>
       </c>
       <c r="D24">
-        <v>2.193E-05</v>
+        <v>2.1929999999999998E-5</v>
       </c>
       <c r="E24">
-        <v>0.23195076</v>
+        <v>0.23195076000000001</v>
       </c>
       <c r="F24">
         <v>145</v>
       </c>
       <c r="G24" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B25">
         <v>4</v>
       </c>
       <c r="C25">
-        <v>0.2417798</v>
+        <v>0.24177979999999999</v>
       </c>
       <c r="D25">
-        <v>5.507E-05</v>
+        <v>5.507E-5</v>
       </c>
       <c r="E25">
-        <v>0.24183487</v>
+        <v>0.24183487000000001</v>
       </c>
       <c r="F25">
         <v>145</v>
       </c>
       <c r="G25" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B26">
         <v>6</v>
@@ -1023,21 +1079,21 @@
         <v>0.24710989</v>
       </c>
       <c r="D26">
-        <v>3.004E-05</v>
+        <v>3.004E-5</v>
       </c>
       <c r="E26">
-        <v>0.24713993</v>
+        <v>0.24713993000000001</v>
       </c>
       <c r="F26">
         <v>145</v>
       </c>
       <c r="G26" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B27">
         <v>8</v>
@@ -1046,21 +1102,21 @@
         <v>0.26431704</v>
       </c>
       <c r="D27">
-        <v>9.584E-05</v>
+        <v>9.5840000000000004E-5</v>
       </c>
       <c r="E27">
-        <v>0.26441288</v>
+        <v>0.26441288000000002</v>
       </c>
       <c r="F27">
         <v>145</v>
       </c>
       <c r="G27" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B28">
         <v>10</v>
@@ -1069,21 +1125,21 @@
         <v>0.27592802</v>
       </c>
       <c r="D28">
-        <v>0.00033617</v>
+        <v>3.3617E-4</v>
       </c>
       <c r="E28">
-        <v>0.27626419</v>
+        <v>0.27626419000000002</v>
       </c>
       <c r="F28">
         <v>145</v>
       </c>
       <c r="G28" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B29">
         <v>12</v>
@@ -1092,136 +1148,136 @@
         <v>0.28126001</v>
       </c>
       <c r="D29">
-        <v>5.293E-05</v>
+        <v>5.2930000000000003E-5</v>
       </c>
       <c r="E29">
-        <v>0.28131294</v>
+        <v>0.28131294000000001</v>
       </c>
       <c r="F29">
         <v>145</v>
       </c>
       <c r="G29" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30">
-        <v>0.22884798</v>
+        <v>0.22884798000000001</v>
       </c>
       <c r="D30">
-        <v>6.198999999999999E-05</v>
+        <v>6.1989999999999994E-5</v>
       </c>
       <c r="E30">
-        <v>0.22890997</v>
+        <v>0.22890996999999999</v>
       </c>
       <c r="F30">
         <v>155</v>
       </c>
       <c r="G30" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B31">
         <v>2</v>
       </c>
       <c r="C31">
-        <v>0.23245382</v>
+        <v>0.23245382000000001</v>
       </c>
       <c r="D31">
-        <v>4.411E-05</v>
+        <v>4.4110000000000003E-5</v>
       </c>
       <c r="E31">
-        <v>0.23249793</v>
+        <v>0.23249792999999999</v>
       </c>
       <c r="F31">
         <v>155</v>
       </c>
       <c r="G31" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B32">
         <v>4</v>
       </c>
       <c r="C32">
-        <v>0.24229002</v>
+        <v>0.24229001999999999</v>
       </c>
       <c r="D32">
-        <v>3.719E-05</v>
+        <v>3.7190000000000001E-5</v>
       </c>
       <c r="E32">
-        <v>0.24232721</v>
+        <v>0.24232720999999999</v>
       </c>
       <c r="F32">
         <v>155</v>
       </c>
       <c r="G32" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B33">
         <v>6</v>
       </c>
       <c r="C33">
-        <v>0.251297</v>
+        <v>0.25129699999999999</v>
       </c>
       <c r="D33">
-        <v>5.722E-05</v>
+        <v>5.7219999999999998E-5</v>
       </c>
       <c r="E33">
-        <v>0.25135422</v>
+        <v>0.25135422000000002</v>
       </c>
       <c r="F33">
         <v>155</v>
       </c>
       <c r="G33" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B34">
         <v>8</v>
       </c>
       <c r="C34">
-        <v>0.26070309</v>
+        <v>0.26070309000000003</v>
       </c>
       <c r="D34">
-        <v>0.00010896</v>
+        <v>1.0896E-4</v>
       </c>
       <c r="E34">
-        <v>0.26081205</v>
+        <v>0.26081205000000002</v>
       </c>
       <c r="F34">
         <v>155</v>
       </c>
       <c r="G34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B35">
         <v>10</v>
@@ -1230,21 +1286,21 @@
         <v>0.27315307</v>
       </c>
       <c r="D35">
-        <v>0.000103</v>
+        <v>1.03E-4</v>
       </c>
       <c r="E35">
-        <v>0.27325607</v>
+        <v>0.27325607000000002</v>
       </c>
       <c r="F35">
         <v>155</v>
       </c>
       <c r="G35" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B36">
         <v>12</v>
@@ -1253,7 +1309,7 @@
         <v>0.28310299</v>
       </c>
       <c r="D36">
-        <v>0.00026703</v>
+        <v>2.6703000000000002E-4</v>
       </c>
       <c r="E36">
         <v>0.28337002</v>
@@ -1262,24 +1318,24 @@
         <v>155</v>
       </c>
       <c r="G36" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B37">
         <v>1</v>
       </c>
       <c r="C37">
-        <v>0.22371292</v>
+        <v>0.22371292000000001</v>
       </c>
       <c r="D37">
-        <v>0.00020289</v>
+        <v>2.0289E-4</v>
       </c>
       <c r="E37">
-        <v>0.22391581</v>
+        <v>0.22391580999999999</v>
       </c>
       <c r="F37">
         <v>171</v>
@@ -1290,19 +1346,19 @@
     </row>
     <row r="38" spans="1:7">
       <c r="A38" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B38">
         <v>2</v>
       </c>
       <c r="C38">
-        <v>0.2283051</v>
+        <v>0.22830510000000001</v>
       </c>
       <c r="D38">
-        <v>0.00013399</v>
+        <v>1.3399000000000001E-4</v>
       </c>
       <c r="E38">
-        <v>0.22843909</v>
+        <v>0.22843909000000001</v>
       </c>
       <c r="F38">
         <v>171</v>
@@ -1313,7 +1369,7 @@
     </row>
     <row r="39" spans="1:7">
       <c r="A39" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B39">
         <v>4</v>
@@ -1322,7 +1378,7 @@
         <v>0.23819208</v>
       </c>
       <c r="D39">
-        <v>0.00010109</v>
+        <v>1.0109E-4</v>
       </c>
       <c r="E39">
         <v>0.23829317</v>
@@ -1336,19 +1392,19 @@
     </row>
     <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B40">
         <v>6</v>
       </c>
       <c r="C40">
-        <v>0.25589895</v>
+        <v>0.25589895000000001</v>
       </c>
       <c r="D40">
-        <v>0.00025511</v>
+        <v>2.5511000000000002E-4</v>
       </c>
       <c r="E40">
-        <v>0.25615406</v>
+        <v>0.25615406000000002</v>
       </c>
       <c r="F40">
         <v>171</v>
@@ -1359,19 +1415,19 @@
     </row>
     <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B41">
         <v>8</v>
       </c>
       <c r="C41">
-        <v>0.26345611</v>
+        <v>0.26345611000000002</v>
       </c>
       <c r="D41">
-        <v>0.00036001</v>
+        <v>3.6001000000000002E-4</v>
       </c>
       <c r="E41">
-        <v>0.26381612</v>
+        <v>0.26381611999999999</v>
       </c>
       <c r="F41">
         <v>171</v>
@@ -1382,19 +1438,19 @@
     </row>
     <row r="42" spans="1:7">
       <c r="A42" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B42">
         <v>10</v>
       </c>
       <c r="C42">
-        <v>0.2758441</v>
+        <v>0.27584409999999998</v>
       </c>
       <c r="D42">
-        <v>0.00015807</v>
+        <v>1.5807000000000001E-4</v>
       </c>
       <c r="E42">
-        <v>0.27600217</v>
+        <v>0.27600216999999999</v>
       </c>
       <c r="F42">
         <v>171</v>
@@ -1405,19 +1461,19 @@
     </row>
     <row r="43" spans="1:7">
       <c r="A43" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B43">
         <v>12</v>
       </c>
       <c r="C43">
-        <v>0.28088808</v>
+        <v>0.28088807999999998</v>
       </c>
       <c r="D43">
-        <v>0.00011897</v>
+        <v>1.1896999999999999E-4</v>
       </c>
       <c r="E43">
-        <v>0.28100705</v>
+        <v>0.28100704999999998</v>
       </c>
       <c r="F43">
         <v>171</v>
@@ -1428,7 +1484,7 @@
     </row>
     <row r="44" spans="1:7">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B44">
         <v>1</v>
@@ -1437,7 +1493,7 @@
         <v>0.22709203</v>
       </c>
       <c r="D44">
-        <v>0.0013299</v>
+        <v>1.3299E-3</v>
       </c>
       <c r="E44">
         <v>0.22842193</v>
@@ -1446,145 +1502,145 @@
         <v>207</v>
       </c>
       <c r="G44" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="45" spans="1:7">
       <c r="A45" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B45">
         <v>2</v>
       </c>
       <c r="C45">
-        <v>0.22897005</v>
+        <v>0.22897005000000001</v>
       </c>
       <c r="D45">
-        <v>0.00070286</v>
+        <v>7.0286000000000003E-4</v>
       </c>
       <c r="E45">
-        <v>0.22967291</v>
+        <v>0.22967291000000001</v>
       </c>
       <c r="F45">
         <v>207</v>
       </c>
       <c r="G45" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" spans="1:7">
       <c r="A46" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B46">
         <v>4</v>
       </c>
       <c r="C46">
-        <v>0.24085879</v>
+        <v>0.24085878999999999</v>
       </c>
       <c r="D46">
-        <v>0.00063491</v>
+        <v>6.3491000000000003E-4</v>
       </c>
       <c r="E46">
-        <v>0.2414937</v>
+        <v>0.24149370000000001</v>
       </c>
       <c r="F46">
         <v>207</v>
       </c>
       <c r="G46" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="47" spans="1:7">
       <c r="A47" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B47">
         <v>6</v>
       </c>
       <c r="C47">
-        <v>0.24863005</v>
+        <v>0.24863004999999999</v>
       </c>
       <c r="D47">
-        <v>0.00064301</v>
+        <v>6.4300999999999996E-4</v>
       </c>
       <c r="E47">
-        <v>0.24927306</v>
+        <v>0.24927305999999999</v>
       </c>
       <c r="F47">
         <v>207</v>
       </c>
       <c r="G47" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B48">
         <v>8</v>
       </c>
       <c r="C48">
-        <v>0.25966501</v>
+        <v>0.25966500999999997</v>
       </c>
       <c r="D48">
-        <v>0.00061488</v>
+        <v>6.1488000000000005E-4</v>
       </c>
       <c r="E48">
-        <v>0.26027989</v>
+        <v>0.26027989000000001</v>
       </c>
       <c r="F48">
         <v>207</v>
       </c>
       <c r="G48" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="49" spans="1:7">
       <c r="A49" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B49">
         <v>10</v>
       </c>
       <c r="C49">
-        <v>0.27248192</v>
+        <v>0.27248191999999999</v>
       </c>
       <c r="D49">
-        <v>0.00067401</v>
+        <v>6.7400999999999995E-4</v>
       </c>
       <c r="E49">
-        <v>0.27315593</v>
+        <v>0.27315592999999999</v>
       </c>
       <c r="F49">
         <v>207</v>
       </c>
       <c r="G49" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="50" spans="1:7">
       <c r="A50" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B50">
         <v>12</v>
       </c>
       <c r="C50">
-        <v>0.28281188</v>
+        <v>0.28281188000000002</v>
       </c>
       <c r="D50">
-        <v>0.00070119</v>
+        <v>7.0118999999999997E-4</v>
       </c>
       <c r="E50">
-        <v>0.28351307</v>
+        <v>0.28351306999999998</v>
       </c>
       <c r="F50">
         <v>207</v>
       </c>
       <c r="G50" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>